<commit_message>
only add afforestation CDR with ecoinvent 3.11 and up
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-carbon-capture.xlsx
+++ b/premise/data/additional_inventories/lci-carbon-capture.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/premise/premise/data/additional_inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFEC7685-3449-6B40-86FB-B8FF4FEF99CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7930783-60D7-7540-BB1A-7ECFB40059AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3085" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3021" uniqueCount="351">
   <si>
     <t>database</t>
   </si>
@@ -1006,12 +1006,6 @@
     <t>For condensing or cooling (varies by setup)</t>
   </si>
   <si>
-    <t>market for methyldiethanolamine</t>
-  </si>
-  <si>
-    <t>methyldiethanolamine</t>
-  </si>
-  <si>
     <t>MDEA make-up for solvent degradation or blowdown, normalized from Antonini et al. (2020) SI LCA workbook: 1.742412e-6 kg solvent proxy per MJ H2 / 0.051247425 kg CO2 stored per MJ H2 = 3.4e-5 kg/kg CO2. The SI uses a diethanolamine market as proxy; this inventory keeps methyldiethanolamine to match the MDEA process chemistry.</t>
   </si>
   <si>
@@ -1049,27 +1043,6 @@
   </si>
   <si>
     <t>Permanent storage of 1 kg non-fossil CO2 from cement flue gas; fossil CO2 co-capture is ignored in this CDR variant.</t>
-  </si>
-  <si>
-    <t>carbon dioxide, captured and stored, by re/afforestation, eucalyptus</t>
-  </si>
-  <si>
-    <t>Simple datasets that models the capture and sequestration of 1 kg of atmopsheric CO2 in biomass.</t>
-  </si>
-  <si>
-    <t>hardwood forestry, eucalyptus ssp., planted forest management</t>
-  </si>
-  <si>
-    <t>cleft timber, green, measured as dry mass</t>
-  </si>
-  <si>
-    <t>carbon dioxide, captured and stored, by re/afforestation, willow</t>
-  </si>
-  <si>
-    <t>willow production, short rotation coppice</t>
-  </si>
-  <si>
-    <t>wood chips and particles, willow, dry, measured as dry mass</t>
   </si>
   <si>
     <t>carbon dioxide, captured, with a solvent-based direct air capture system, 1MtCO2, with hydrogen heat, and grid electricity</t>
@@ -1112,7 +1085,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="0.0E+00"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
@@ -1121,7 +1094,6 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="_ * #,##0.0000_ ;_ * \-#,##0.0000_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="170" formatCode="0.00000"/>
-    <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -1243,7 +1215,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1284,7 +1256,6 @@
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="170" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1608,7 +1579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V773"/>
+  <dimension ref="A1:V772"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="47.33203125" customWidth="1"/>
@@ -12782,13 +12753,13 @@
     </row>
     <row r="624" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A624" s="15" t="s">
-        <v>326</v>
+        <v>184</v>
       </c>
       <c r="B624">
         <v>3.4E-5</v>
       </c>
       <c r="C624" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="D624" t="s">
         <v>10</v>
@@ -12797,10 +12768,10 @@
         <v>28</v>
       </c>
       <c r="G624" s="15" t="s">
-        <v>327</v>
+        <v>185</v>
       </c>
       <c r="H624" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I624">
         <v>0</v>
@@ -12827,7 +12798,7 @@
         <v>79</v>
       </c>
       <c r="H625" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="626" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -12850,7 +12821,7 @@
         <v>81</v>
       </c>
       <c r="H626" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="627" spans="1:13" x14ac:dyDescent="0.2">
@@ -12893,7 +12864,7 @@
         <v>61</v>
       </c>
       <c r="H628" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="629" spans="1:13" x14ac:dyDescent="0.2">
@@ -12916,7 +12887,7 @@
         <v>0</v>
       </c>
       <c r="H629" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="631" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -12924,7 +12895,7 @@
         <v>2</v>
       </c>
       <c r="B631" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="632" spans="1:13" x14ac:dyDescent="0.2">
@@ -12972,7 +12943,7 @@
         <v>15</v>
       </c>
       <c r="B637" s="6" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="638" spans="1:13" x14ac:dyDescent="0.2">
@@ -12980,7 +12951,7 @@
         <v>13</v>
       </c>
       <c r="B638" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="639" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -13031,7 +13002,7 @@
     </row>
     <row r="641" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A641" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B641">
         <v>1</v>
@@ -13069,7 +13040,7 @@
         <v>61</v>
       </c>
       <c r="H642" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="643" spans="1:22" x14ac:dyDescent="0.2">
@@ -13089,7 +13060,7 @@
         <v>57</v>
       </c>
       <c r="H643" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="645" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -13097,7 +13068,7 @@
         <v>2</v>
       </c>
       <c r="B645" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C645" s="37"/>
       <c r="D645" s="37"/>
@@ -13293,7 +13264,7 @@
         <v>13</v>
       </c>
       <c r="B652" s="37" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C652" s="37"/>
       <c r="D652" s="37"/>
@@ -13384,7 +13355,7 @@
     </row>
     <row r="655" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A655" s="28" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B655" s="34">
         <v>1</v>
@@ -13847,7 +13818,7 @@
       </c>
       <c r="G667" s="29"/>
       <c r="H667" s="37" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="I667" s="37"/>
       <c r="J667" s="37"/>
@@ -13892,850 +13863,668 @@
       <c r="A669" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B669" s="5" t="s">
+      <c r="B669" s="1" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="670" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A670" t="s">
+        <v>4</v>
+      </c>
+      <c r="B670">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="671" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A671" t="s">
+        <v>5</v>
+      </c>
+      <c r="B671" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="672" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A672" t="s">
+        <v>7</v>
+      </c>
+      <c r="B672" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="673" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A673" t="s">
+        <v>9</v>
+      </c>
+      <c r="B673" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="674" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A674" t="s">
+        <v>11</v>
+      </c>
+      <c r="B674" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="675" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A675" t="s">
+        <v>13</v>
+      </c>
+      <c r="B675" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="676" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A676" t="s">
+        <v>15</v>
+      </c>
+      <c r="B676" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="677" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A677" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="678" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A678" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B678" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C678" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D678" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E678" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F678" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G678" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H678" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I678" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J678" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K678" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L678" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M678" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="679" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A679" t="s">
+        <v>339</v>
+      </c>
+      <c r="B679">
+        <v>1</v>
+      </c>
+      <c r="C679" t="s">
+        <v>12</v>
+      </c>
+      <c r="D679" t="s">
+        <v>10</v>
+      </c>
+      <c r="F679" t="s">
+        <v>26</v>
+      </c>
+      <c r="G679" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="680" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A680" t="s">
+        <v>27</v>
+      </c>
+      <c r="B680">
+        <v>5.0000000000000002E-11</v>
+      </c>
+      <c r="C680" t="s">
+        <v>12</v>
+      </c>
+      <c r="D680" t="s">
+        <v>9</v>
+      </c>
+      <c r="F680" t="s">
+        <v>28</v>
+      </c>
+      <c r="G680" t="s">
+        <v>29</v>
+      </c>
+      <c r="H680" t="s">
+        <v>30</v>
+      </c>
+      <c r="I680">
+        <v>5</v>
+      </c>
+      <c r="J680" s="38">
+        <v>5.0000000000000002E-11</v>
+      </c>
+      <c r="K680" s="38">
+        <v>3.9999999999999998E-11</v>
+      </c>
+      <c r="L680" s="38">
+        <v>6.6666666666666669E-11</v>
+      </c>
+    </row>
+    <row r="681" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A681" t="s">
+        <v>31</v>
+      </c>
+      <c r="B681">
+        <v>-5.0000000000000002E-11</v>
+      </c>
+      <c r="C681" t="s">
+        <v>12</v>
+      </c>
+      <c r="D681" t="s">
+        <v>9</v>
+      </c>
+      <c r="F681" t="s">
+        <v>28</v>
+      </c>
+      <c r="G681" t="s">
+        <v>29</v>
+      </c>
+      <c r="H681" t="s">
+        <v>32</v>
+      </c>
+      <c r="I681">
+        <v>5</v>
+      </c>
+      <c r="J681">
+        <v>-5.0000000000000002E-11</v>
+      </c>
+      <c r="K681" s="38">
+        <v>-6.6666666666666669E-11</v>
+      </c>
+      <c r="L681" s="38">
+        <v>-3.9999999999999998E-11</v>
+      </c>
+      <c r="M681" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="682" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A682" t="s">
+        <v>33</v>
+      </c>
+      <c r="B682">
+        <v>3.4369999999999998</v>
+      </c>
+      <c r="C682" t="s">
+        <v>34</v>
+      </c>
+      <c r="D682" t="s">
+        <v>10</v>
+      </c>
+      <c r="F682" t="s">
+        <v>28</v>
+      </c>
+      <c r="G682" t="s">
+        <v>35</v>
+      </c>
+      <c r="H682" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="683" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A683" t="s">
+        <v>37</v>
+      </c>
+      <c r="B683">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="C683" t="s">
+        <v>38</v>
+      </c>
+      <c r="D683" t="s">
+        <v>10</v>
+      </c>
+      <c r="F683" t="s">
+        <v>28</v>
+      </c>
+      <c r="G683" t="s">
+        <v>39</v>
+      </c>
+      <c r="H683" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="684" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A684" s="39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B684">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="C684" t="s">
+        <v>41</v>
+      </c>
+      <c r="D684" t="s">
+        <v>10</v>
+      </c>
+      <c r="F684" t="s">
+        <v>28</v>
+      </c>
+      <c r="G684" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="H684" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="685" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A685" t="s">
+        <v>43</v>
+      </c>
+      <c r="B685" s="40">
+        <v>-4.0000000000000001E-3</v>
+      </c>
+      <c r="C685" t="s">
+        <v>34</v>
+      </c>
+      <c r="D685" t="s">
+        <v>10</v>
+      </c>
+      <c r="F685" t="s">
+        <v>28</v>
+      </c>
+      <c r="G685" t="s">
+        <v>44</v>
+      </c>
+      <c r="H685" s="41" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="686" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A686" t="s">
+        <v>45</v>
+      </c>
+      <c r="B686" s="42">
+        <v>-3.5000000000000001E-3</v>
+      </c>
+      <c r="C686" t="s">
+        <v>41</v>
+      </c>
+      <c r="D686" t="s">
+        <v>10</v>
+      </c>
+      <c r="F686" t="s">
+        <v>28</v>
+      </c>
+      <c r="G686" t="s">
+        <v>46</v>
+      </c>
+      <c r="H686" s="41" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="687" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A687" t="s">
+        <v>47</v>
+      </c>
+      <c r="B687">
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="C687" t="s">
+        <v>12</v>
+      </c>
+      <c r="D687" t="s">
+        <v>48</v>
+      </c>
+      <c r="F687" t="s">
+        <v>28</v>
+      </c>
+      <c r="G687" t="s">
+        <v>49</v>
+      </c>
+      <c r="H687" t="s">
+        <v>50</v>
+      </c>
+      <c r="I687">
+        <v>5</v>
+      </c>
+      <c r="J687">
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="K687">
+        <v>0.33</v>
+      </c>
+      <c r="L687">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="688" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A688" t="s">
         <v>341</v>
       </c>
-      <c r="C669" s="37"/>
-      <c r="D669" s="37"/>
-      <c r="E669" s="37"/>
-      <c r="F669" s="37"/>
-      <c r="G669" s="37"/>
-      <c r="H669" s="37"/>
-      <c r="I669" s="37"/>
-      <c r="J669" s="37"/>
-      <c r="K669" s="37"/>
-      <c r="L669" s="37"/>
-      <c r="M669" s="37"/>
-      <c r="N669" s="37"/>
-      <c r="O669" s="37"/>
-      <c r="P669" s="37"/>
-      <c r="Q669" s="37"/>
-      <c r="R669" s="37"/>
-      <c r="S669" s="37"/>
-      <c r="T669" s="37"/>
-      <c r="U669" s="37"/>
-      <c r="V669" s="37"/>
-    </row>
-    <row r="670" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A670" s="37" t="s">
+      <c r="B688">
+        <v>8.4999999999999992E-2</v>
+      </c>
+      <c r="C688" t="s">
+        <v>12</v>
+      </c>
+      <c r="D688" t="s">
+        <v>10</v>
+      </c>
+      <c r="F688" t="s">
+        <v>28</v>
+      </c>
+      <c r="G688" t="s">
+        <v>342</v>
+      </c>
+      <c r="H688" t="s">
+        <v>343</v>
+      </c>
+      <c r="I688">
+        <v>5</v>
+      </c>
+      <c r="J688">
+        <v>8.4999999999999992E-2</v>
+      </c>
+      <c r="K688">
+        <v>8.4999999999999992E-2</v>
+      </c>
+      <c r="L688">
+        <v>0.1127777777777778</v>
+      </c>
+    </row>
+    <row r="689" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A689" t="s">
+        <v>55</v>
+      </c>
+      <c r="B689">
+        <v>1</v>
+      </c>
+      <c r="D689" t="s">
+        <v>10</v>
+      </c>
+      <c r="E689" t="s">
+        <v>56</v>
+      </c>
+      <c r="F689" t="s">
+        <v>57</v>
+      </c>
+      <c r="H689" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="691" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A691" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B691" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="692" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A692" t="s">
+        <v>4</v>
+      </c>
+      <c r="B692">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="693" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A693" t="s">
+        <v>5</v>
+      </c>
+      <c r="B693" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="694" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A694" t="s">
+        <v>7</v>
+      </c>
+      <c r="B694" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="695" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A695" t="s">
+        <v>9</v>
+      </c>
+      <c r="B695" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="696" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A696" t="s">
         <v>11</v>
       </c>
-      <c r="B670" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="C670" s="37"/>
-      <c r="D670" s="37"/>
-      <c r="E670" s="37"/>
-      <c r="F670" s="37"/>
-      <c r="G670" s="37"/>
-      <c r="H670" s="37"/>
-      <c r="I670" s="37"/>
-      <c r="J670" s="37"/>
-      <c r="K670" s="37"/>
-      <c r="L670" s="37"/>
-      <c r="M670" s="37"/>
-      <c r="N670" s="37"/>
-      <c r="O670" s="37"/>
-      <c r="P670" s="37"/>
-      <c r="Q670" s="37"/>
-      <c r="R670" s="37"/>
-      <c r="S670" s="37"/>
-      <c r="T670" s="37"/>
-      <c r="U670" s="37"/>
-      <c r="V670" s="37"/>
-    </row>
-    <row r="671" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A671" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B671" s="37">
+      <c r="B696" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="697" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A697" t="s">
+        <v>13</v>
+      </c>
+      <c r="B697" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="698" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A698" t="s">
+        <v>15</v>
+      </c>
+      <c r="B698" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="699" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A699" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="700" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A700" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B700" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C700" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D700" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E700" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F700" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G700" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H700" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I700" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J700" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K700" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L700" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M700" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="701" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A701" t="s">
+        <v>344</v>
+      </c>
+      <c r="B701">
         <v>1</v>
       </c>
-      <c r="C671" s="37"/>
-      <c r="D671" s="37"/>
-      <c r="E671" s="37"/>
-      <c r="F671" s="37"/>
-      <c r="G671" s="37"/>
-      <c r="H671" s="37"/>
-      <c r="I671" s="37"/>
-      <c r="J671" s="37"/>
-      <c r="K671" s="37"/>
-      <c r="L671" s="37"/>
-      <c r="M671" s="37"/>
-      <c r="N671" s="37"/>
-      <c r="O671" s="37"/>
-      <c r="P671" s="37"/>
-      <c r="Q671" s="37"/>
-      <c r="R671" s="37"/>
-      <c r="S671" s="37"/>
-      <c r="T671" s="37"/>
-      <c r="U671" s="37"/>
-      <c r="V671" s="37"/>
-    </row>
-    <row r="672" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A672" s="37" t="s">
+      <c r="C701" t="s">
+        <v>12</v>
+      </c>
+      <c r="D701" t="s">
+        <v>10</v>
+      </c>
+      <c r="F701" t="s">
+        <v>26</v>
+      </c>
+      <c r="G701" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="702" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A702" t="s">
+        <v>27</v>
+      </c>
+      <c r="B702">
+        <v>5.0000000000000002E-11</v>
+      </c>
+      <c r="C702" t="s">
+        <v>12</v>
+      </c>
+      <c r="D702" t="s">
+        <v>9</v>
+      </c>
+      <c r="F702" t="s">
+        <v>28</v>
+      </c>
+      <c r="G702" t="s">
+        <v>29</v>
+      </c>
+      <c r="H702" t="s">
+        <v>30</v>
+      </c>
+      <c r="I702">
         <v>5</v>
       </c>
-      <c r="B672" s="37" t="s">
-        <v>6</v>
-      </c>
-      <c r="C672" s="37"/>
-      <c r="D672" s="37"/>
-      <c r="E672" s="37"/>
-      <c r="F672" s="37"/>
-      <c r="G672" s="37"/>
-      <c r="H672" s="37"/>
-      <c r="I672" s="37"/>
-      <c r="J672" s="37"/>
-      <c r="K672" s="37"/>
-      <c r="L672" s="37"/>
-      <c r="M672" s="37"/>
-      <c r="N672" s="37"/>
-      <c r="O672" s="37"/>
-      <c r="P672" s="37"/>
-      <c r="Q672" s="37"/>
-      <c r="R672" s="37"/>
-      <c r="S672" s="37"/>
-      <c r="T672" s="37"/>
-      <c r="U672" s="37"/>
-      <c r="V672" s="37"/>
-    </row>
-    <row r="673" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A673" s="37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B673" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="C673" s="37"/>
-      <c r="D673" s="37"/>
-      <c r="E673" s="37"/>
-      <c r="F673" s="37"/>
-      <c r="G673" s="37"/>
-      <c r="H673" s="37"/>
-      <c r="I673" s="37"/>
-      <c r="J673" s="37"/>
-      <c r="K673" s="37"/>
-      <c r="L673" s="37"/>
-      <c r="M673" s="37"/>
-      <c r="N673" s="37"/>
-      <c r="O673" s="37"/>
-      <c r="P673" s="37"/>
-      <c r="Q673" s="37"/>
-      <c r="R673" s="37"/>
-      <c r="S673" s="37"/>
-      <c r="T673" s="37"/>
-      <c r="U673" s="37"/>
-      <c r="V673" s="37"/>
-    </row>
-    <row r="674" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A674" s="37" t="s">
+      <c r="J702" s="38">
+        <v>5.0000000000000002E-11</v>
+      </c>
+      <c r="K702" s="38">
+        <v>3.9999999999999998E-11</v>
+      </c>
+      <c r="L702" s="38">
+        <v>6.6666666666666669E-11</v>
+      </c>
+    </row>
+    <row r="703" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A703" t="s">
+        <v>31</v>
+      </c>
+      <c r="B703">
+        <v>-5.0000000000000002E-11</v>
+      </c>
+      <c r="C703" t="s">
+        <v>12</v>
+      </c>
+      <c r="D703" t="s">
         <v>9</v>
       </c>
-      <c r="B674" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="C674" s="37"/>
-      <c r="D674" s="37"/>
-      <c r="E674" s="37"/>
-      <c r="F674" s="37"/>
-      <c r="G674" s="37"/>
-      <c r="H674" s="37"/>
-      <c r="I674" s="37"/>
-      <c r="J674" s="37"/>
-      <c r="K674" s="37"/>
-      <c r="L674" s="37"/>
-      <c r="M674" s="37"/>
-      <c r="N674" s="37"/>
-      <c r="O674" s="37"/>
-      <c r="P674" s="37"/>
-      <c r="Q674" s="37"/>
-      <c r="R674" s="37"/>
-      <c r="S674" s="37"/>
-      <c r="T674" s="37"/>
-      <c r="U674" s="37"/>
-      <c r="V674" s="37"/>
-    </row>
-    <row r="675" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A675" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="B675" t="s">
-        <v>342</v>
-      </c>
-      <c r="C675" s="37"/>
-      <c r="D675" s="37"/>
-      <c r="E675" s="37"/>
-      <c r="F675" s="37"/>
-      <c r="G675" s="37"/>
-      <c r="H675" s="37"/>
-      <c r="I675" s="37"/>
-      <c r="J675" s="37"/>
-      <c r="K675" s="37"/>
-      <c r="L675" s="37"/>
-      <c r="M675" s="37"/>
-      <c r="N675" s="37"/>
-      <c r="O675" s="37"/>
-      <c r="P675" s="37"/>
-      <c r="Q675" s="37"/>
-      <c r="R675" s="37"/>
-      <c r="S675" s="37"/>
-      <c r="T675" s="37"/>
-      <c r="U675" s="37"/>
-      <c r="V675" s="37"/>
-    </row>
-    <row r="676" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A676" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="B676" s="37"/>
-      <c r="C676" s="37"/>
-      <c r="D676" s="37"/>
-      <c r="E676" s="37"/>
-      <c r="F676" s="37"/>
-      <c r="G676" s="37"/>
-      <c r="H676" s="37"/>
-      <c r="I676" s="37"/>
-      <c r="J676" s="37"/>
-      <c r="K676" s="37"/>
-      <c r="L676" s="37"/>
-      <c r="M676" s="37"/>
-      <c r="N676" s="37"/>
-      <c r="O676" s="37"/>
-      <c r="P676" s="37"/>
-      <c r="Q676" s="37"/>
-      <c r="R676" s="37"/>
-      <c r="S676" s="37"/>
-      <c r="T676" s="37"/>
-      <c r="U676" s="37"/>
-      <c r="V676" s="37"/>
-    </row>
-    <row r="677" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A677" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B677" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C677" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D677" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E677" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F677" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G677" s="5" t="s">
+      <c r="F703" t="s">
+        <v>28</v>
+      </c>
+      <c r="G703" t="s">
+        <v>29</v>
+      </c>
+      <c r="H703" t="s">
+        <v>32</v>
+      </c>
+      <c r="I703">
         <v>5</v>
       </c>
-      <c r="H677" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I677" s="5"/>
-      <c r="J677" s="5"/>
-      <c r="K677" s="5"/>
-      <c r="L677" s="5"/>
-      <c r="M677" s="5"/>
-      <c r="N677" s="5"/>
-      <c r="O677" s="5"/>
-      <c r="P677" s="5"/>
-      <c r="Q677" s="5"/>
-      <c r="R677" s="5"/>
-      <c r="S677" s="5"/>
-      <c r="T677" s="37"/>
-      <c r="U677" s="37"/>
-      <c r="V677" s="37"/>
-    </row>
-    <row r="678" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A678" s="28" t="s">
-        <v>341</v>
-      </c>
-      <c r="B678" s="38">
+      <c r="J703" s="38">
+        <v>-5.0000000000000002E-11</v>
+      </c>
+      <c r="K703" s="38">
+        <v>-6.6666666666666669E-11</v>
+      </c>
+      <c r="L703" s="38">
+        <v>-3.9999999999999998E-11</v>
+      </c>
+      <c r="M703" t="b">
         <v>1</v>
       </c>
-      <c r="C678" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="D678" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="E678" s="37"/>
-      <c r="F678" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="G678" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="H678" s="37"/>
-      <c r="I678" s="37"/>
-      <c r="J678" s="37"/>
-      <c r="K678" s="37"/>
-      <c r="L678" s="37"/>
-      <c r="M678" s="37"/>
-      <c r="N678" s="37"/>
-      <c r="O678" s="37"/>
-      <c r="P678" s="37"/>
-      <c r="Q678" s="37"/>
-      <c r="R678" s="37"/>
-      <c r="S678" s="37"/>
-      <c r="T678" s="37"/>
-      <c r="U678" s="37"/>
-      <c r="V678" s="37"/>
-    </row>
-    <row r="679" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A679" t="s">
-        <v>343</v>
-      </c>
-      <c r="B679">
-        <v>0.7407407407407407</v>
-      </c>
-      <c r="C679" t="s">
-        <v>74</v>
-      </c>
-      <c r="D679" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F679" t="s">
-        <v>28</v>
-      </c>
-      <c r="G679" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="681" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A681" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B681" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="C681" s="37"/>
-      <c r="D681" s="37"/>
-      <c r="E681" s="37"/>
-      <c r="F681" s="37"/>
-      <c r="G681" s="37"/>
-      <c r="H681" s="37"/>
-      <c r="I681" s="37"/>
-      <c r="J681" s="37"/>
-      <c r="K681" s="37"/>
-      <c r="L681" s="37"/>
-      <c r="M681" s="37"/>
-      <c r="N681" s="37"/>
-      <c r="O681" s="37"/>
-      <c r="P681" s="37"/>
-      <c r="Q681" s="37"/>
-      <c r="R681" s="37"/>
-      <c r="S681" s="37"/>
-      <c r="T681" s="37"/>
-      <c r="U681" s="37"/>
-      <c r="V681" s="37"/>
-    </row>
-    <row r="682" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A682" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="B682" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="C682" s="37"/>
-      <c r="D682" s="37"/>
-      <c r="E682" s="37"/>
-      <c r="F682" s="37"/>
-      <c r="G682" s="37"/>
-      <c r="H682" s="37"/>
-      <c r="I682" s="37"/>
-      <c r="J682" s="37"/>
-      <c r="K682" s="37"/>
-      <c r="L682" s="37"/>
-      <c r="M682" s="37"/>
-      <c r="N682" s="37"/>
-      <c r="O682" s="37"/>
-      <c r="P682" s="37"/>
-      <c r="Q682" s="37"/>
-      <c r="R682" s="37"/>
-      <c r="S682" s="37"/>
-      <c r="T682" s="37"/>
-      <c r="U682" s="37"/>
-      <c r="V682" s="37"/>
-    </row>
-    <row r="683" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A683" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B683" s="37">
-        <v>1</v>
-      </c>
-      <c r="C683" s="37"/>
-      <c r="D683" s="37"/>
-      <c r="E683" s="37"/>
-      <c r="F683" s="37"/>
-      <c r="G683" s="37"/>
-      <c r="H683" s="37"/>
-      <c r="I683" s="37"/>
-      <c r="J683" s="37"/>
-      <c r="K683" s="37"/>
-      <c r="L683" s="37"/>
-      <c r="M683" s="37"/>
-      <c r="N683" s="37"/>
-      <c r="O683" s="37"/>
-      <c r="P683" s="37"/>
-      <c r="Q683" s="37"/>
-      <c r="R683" s="37"/>
-      <c r="S683" s="37"/>
-      <c r="T683" s="37"/>
-      <c r="U683" s="37"/>
-      <c r="V683" s="37"/>
-    </row>
-    <row r="684" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A684" s="37" t="s">
-        <v>5</v>
-      </c>
-      <c r="B684" s="37" t="s">
-        <v>6</v>
-      </c>
-      <c r="C684" s="37"/>
-      <c r="D684" s="37"/>
-      <c r="E684" s="37"/>
-      <c r="F684" s="37"/>
-      <c r="G684" s="37"/>
-      <c r="H684" s="37"/>
-      <c r="I684" s="37"/>
-      <c r="J684" s="37"/>
-      <c r="K684" s="37"/>
-      <c r="L684" s="37"/>
-      <c r="M684" s="37"/>
-      <c r="N684" s="37"/>
-      <c r="O684" s="37"/>
-      <c r="P684" s="37"/>
-      <c r="Q684" s="37"/>
-      <c r="R684" s="37"/>
-      <c r="S684" s="37"/>
-      <c r="T684" s="37"/>
-      <c r="U684" s="37"/>
-      <c r="V684" s="37"/>
-    </row>
-    <row r="685" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A685" s="37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B685" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="C685" s="37"/>
-      <c r="D685" s="37"/>
-      <c r="E685" s="37"/>
-      <c r="F685" s="37"/>
-      <c r="G685" s="37"/>
-      <c r="H685" s="37"/>
-      <c r="I685" s="37"/>
-      <c r="J685" s="37"/>
-      <c r="K685" s="37"/>
-      <c r="L685" s="37"/>
-      <c r="M685" s="37"/>
-      <c r="N685" s="37"/>
-      <c r="O685" s="37"/>
-      <c r="P685" s="37"/>
-      <c r="Q685" s="37"/>
-      <c r="R685" s="37"/>
-      <c r="S685" s="37"/>
-      <c r="T685" s="37"/>
-      <c r="U685" s="37"/>
-      <c r="V685" s="37"/>
-    </row>
-    <row r="686" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A686" s="37" t="s">
-        <v>9</v>
-      </c>
-      <c r="B686" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="C686" s="37"/>
-      <c r="D686" s="37"/>
-      <c r="E686" s="37"/>
-      <c r="F686" s="37"/>
-      <c r="G686" s="37"/>
-      <c r="H686" s="37"/>
-      <c r="I686" s="37"/>
-      <c r="J686" s="37"/>
-      <c r="K686" s="37"/>
-      <c r="L686" s="37"/>
-      <c r="M686" s="37"/>
-      <c r="N686" s="37"/>
-      <c r="O686" s="37"/>
-      <c r="P686" s="37"/>
-      <c r="Q686" s="37"/>
-      <c r="R686" s="37"/>
-      <c r="S686" s="37"/>
-      <c r="T686" s="37"/>
-      <c r="U686" s="37"/>
-      <c r="V686" s="37"/>
-    </row>
-    <row r="687" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A687" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="B687" t="s">
-        <v>342</v>
-      </c>
-      <c r="C687" s="37"/>
-      <c r="D687" s="37"/>
-      <c r="E687" s="37"/>
-      <c r="F687" s="37"/>
-      <c r="G687" s="37"/>
-      <c r="H687" s="37"/>
-      <c r="I687" s="37"/>
-      <c r="J687" s="37"/>
-      <c r="K687" s="37"/>
-      <c r="L687" s="37"/>
-      <c r="M687" s="37"/>
-      <c r="N687" s="37"/>
-      <c r="O687" s="37"/>
-      <c r="P687" s="37"/>
-      <c r="Q687" s="37"/>
-      <c r="R687" s="37"/>
-      <c r="S687" s="37"/>
-      <c r="T687" s="37"/>
-      <c r="U687" s="37"/>
-      <c r="V687" s="37"/>
-    </row>
-    <row r="688" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A688" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="B688" s="37"/>
-      <c r="C688" s="37"/>
-      <c r="D688" s="37"/>
-      <c r="E688" s="37"/>
-      <c r="F688" s="37"/>
-      <c r="G688" s="37"/>
-      <c r="H688" s="37"/>
-      <c r="I688" s="37"/>
-      <c r="J688" s="37"/>
-      <c r="K688" s="37"/>
-      <c r="L688" s="37"/>
-      <c r="M688" s="37"/>
-      <c r="N688" s="37"/>
-      <c r="O688" s="37"/>
-      <c r="P688" s="37"/>
-      <c r="Q688" s="37"/>
-      <c r="R688" s="37"/>
-      <c r="S688" s="37"/>
-      <c r="T688" s="37"/>
-      <c r="U688" s="37"/>
-      <c r="V688" s="37"/>
-    </row>
-    <row r="689" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A689" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B689" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C689" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D689" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E689" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F689" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G689" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H689" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I689" s="5"/>
-      <c r="J689" s="5"/>
-      <c r="K689" s="5"/>
-      <c r="L689" s="5"/>
-      <c r="M689" s="5"/>
-      <c r="N689" s="5"/>
-      <c r="O689" s="5"/>
-      <c r="P689" s="5"/>
-      <c r="Q689" s="5"/>
-      <c r="R689" s="5"/>
-      <c r="S689" s="5"/>
-      <c r="T689" s="37"/>
-      <c r="U689" s="37"/>
-      <c r="V689" s="37"/>
-    </row>
-    <row r="690" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A690" s="28" t="s">
-        <v>345</v>
-      </c>
-      <c r="B690" s="38">
-        <v>1</v>
-      </c>
-      <c r="C690" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="D690" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="E690" s="37"/>
-      <c r="F690" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="G690" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="H690" s="37"/>
-      <c r="I690" s="37"/>
-      <c r="J690" s="37"/>
-      <c r="K690" s="37"/>
-      <c r="L690" s="37"/>
-      <c r="M690" s="37"/>
-      <c r="N690" s="37"/>
-      <c r="O690" s="37"/>
-      <c r="P690" s="37"/>
-      <c r="Q690" s="37"/>
-      <c r="R690" s="37"/>
-      <c r="S690" s="37"/>
-      <c r="T690" s="37"/>
-      <c r="U690" s="37"/>
-      <c r="V690" s="37"/>
-    </row>
-    <row r="691" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A691" t="s">
-        <v>346</v>
-      </c>
-      <c r="B691">
-        <v>0.56818181818181823</v>
-      </c>
-      <c r="C691" t="s">
-        <v>74</v>
-      </c>
-      <c r="D691" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F691" t="s">
-        <v>28</v>
-      </c>
-      <c r="G691" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="693" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A693" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B693" s="1" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="694" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A694" t="s">
-        <v>4</v>
-      </c>
-      <c r="B694">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="695" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A695" t="s">
-        <v>5</v>
-      </c>
-      <c r="B695" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="696" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A696" t="s">
-        <v>7</v>
-      </c>
-      <c r="B696" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="697" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A697" t="s">
-        <v>9</v>
-      </c>
-      <c r="B697" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="698" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A698" t="s">
-        <v>11</v>
-      </c>
-      <c r="B698" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="699" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A699" t="s">
-        <v>13</v>
-      </c>
-      <c r="B699" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="700" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A700" t="s">
-        <v>15</v>
-      </c>
-      <c r="B700" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="701" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A701" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="702" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A702" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B702" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C702" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D702" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E702" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F702" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G702" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H702" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I702" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J702" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K702" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="L702" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M702" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="703" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A703" t="s">
-        <v>348</v>
-      </c>
-      <c r="B703">
-        <v>1</v>
-      </c>
-      <c r="C703" t="s">
-        <v>12</v>
-      </c>
-      <c r="D703" t="s">
-        <v>10</v>
-      </c>
-      <c r="F703" t="s">
-        <v>26</v>
-      </c>
-      <c r="G703" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="704" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="704" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A704" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B704">
-        <v>5.0000000000000002E-11</v>
+        <v>3.4369999999999998</v>
       </c>
       <c r="C704" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="D704" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F704" t="s">
         <v>28</v>
       </c>
       <c r="G704" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H704" t="s">
-        <v>30</v>
-      </c>
-      <c r="I704">
-        <v>5</v>
-      </c>
-      <c r="J704" s="39">
-        <v>5.0000000000000002E-11</v>
-      </c>
-      <c r="K704" s="39">
-        <v>3.9999999999999998E-11</v>
-      </c>
-      <c r="L704" s="39">
-        <v>6.6666666666666669E-11</v>
-      </c>
-    </row>
-    <row r="705" spans="1:13" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="705" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A705" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B705">
-        <v>-5.0000000000000002E-11</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="C705" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="D705" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F705" t="s">
         <v>28</v>
       </c>
       <c r="G705" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="H705" t="s">
-        <v>32</v>
-      </c>
-      <c r="I705">
-        <v>5</v>
-      </c>
-      <c r="J705">
-        <v>-5.0000000000000002E-11</v>
-      </c>
-      <c r="K705" s="39">
-        <v>-6.6666666666666669E-11</v>
-      </c>
-      <c r="L705" s="39">
-        <v>-3.9999999999999998E-11</v>
-      </c>
-      <c r="M705" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="706" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A706" t="s">
-        <v>33</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="706" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A706" s="39" t="s">
+        <v>40</v>
       </c>
       <c r="B706">
-        <v>3.4369999999999998</v>
+        <v>3.5000000000000001E-3</v>
       </c>
       <c r="C706" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D706" t="s">
         <v>10</v>
@@ -14743,22 +14532,22 @@
       <c r="F706" t="s">
         <v>28</v>
       </c>
-      <c r="G706" t="s">
-        <v>35</v>
+      <c r="G706" s="39" t="s">
+        <v>42</v>
       </c>
       <c r="H706" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="707" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="707" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A707" t="s">
-        <v>37</v>
-      </c>
-      <c r="B707">
-        <v>4.0000000000000001E-3</v>
+        <v>43</v>
+      </c>
+      <c r="B707" s="40">
+        <v>-4.0000000000000001E-3</v>
       </c>
       <c r="C707" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D707" t="s">
         <v>10</v>
@@ -14767,18 +14556,18 @@
         <v>28</v>
       </c>
       <c r="G707" t="s">
-        <v>39</v>
-      </c>
-      <c r="H707" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="708" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A708" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="B708">
-        <v>3.5000000000000001E-3</v>
+        <v>44</v>
+      </c>
+      <c r="H707" s="41" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="708" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A708" t="s">
+        <v>45</v>
+      </c>
+      <c r="B708" s="42">
+        <v>-3.5000000000000001E-3</v>
       </c>
       <c r="C708" t="s">
         <v>41</v>
@@ -14789,45 +14578,57 @@
       <c r="F708" t="s">
         <v>28</v>
       </c>
-      <c r="G708" s="40" t="s">
-        <v>42</v>
-      </c>
-      <c r="H708" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="709" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="G708" t="s">
+        <v>46</v>
+      </c>
+      <c r="H708" s="41" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="709" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A709" t="s">
-        <v>43</v>
-      </c>
-      <c r="B709" s="41">
-        <v>-4.0000000000000001E-3</v>
+        <v>47</v>
+      </c>
+      <c r="B709">
+        <v>0.34499999999999997</v>
       </c>
       <c r="C709" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="D709" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="F709" t="s">
         <v>28</v>
       </c>
       <c r="G709" t="s">
-        <v>44</v>
-      </c>
-      <c r="H709" s="42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="710" spans="1:13" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="H709" t="s">
+        <v>50</v>
+      </c>
+      <c r="I709">
+        <v>5</v>
+      </c>
+      <c r="J709">
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="K709">
+        <v>0.33</v>
+      </c>
+      <c r="L709">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="710" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A710" t="s">
-        <v>45</v>
-      </c>
-      <c r="B710" s="43">
-        <v>-3.5000000000000001E-3</v>
+        <v>341</v>
+      </c>
+      <c r="B710">
+        <v>8.4999999999999992E-2</v>
       </c>
       <c r="C710" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D710" t="s">
         <v>10</v>
@@ -14836,238 +14637,238 @@
         <v>28</v>
       </c>
       <c r="G710" t="s">
-        <v>46</v>
-      </c>
-      <c r="H710" s="42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="711" spans="1:13" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+      <c r="H710" t="s">
+        <v>343</v>
+      </c>
+      <c r="I710">
+        <v>5</v>
+      </c>
+      <c r="J710">
+        <v>8.4999999999999992E-2</v>
+      </c>
+      <c r="K710">
+        <v>8.4999999999999992E-2</v>
+      </c>
+      <c r="L710">
+        <v>0.1127777777777778</v>
+      </c>
+    </row>
+    <row r="711" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A711" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B711">
-        <v>0.34499999999999997</v>
+        <v>1</v>
       </c>
       <c r="C711" t="s">
         <v>12</v>
       </c>
       <c r="D711" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="F711" t="s">
         <v>28</v>
       </c>
-      <c r="G711" t="s">
-        <v>49</v>
+      <c r="G711" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="H711" t="s">
-        <v>50</v>
-      </c>
-      <c r="I711">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="712" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A712" t="s">
+        <v>55</v>
+      </c>
+      <c r="B712">
+        <v>1</v>
+      </c>
+      <c r="D712" t="s">
+        <v>10</v>
+      </c>
+      <c r="E712" t="s">
+        <v>56</v>
+      </c>
+      <c r="F712" t="s">
+        <v>57</v>
+      </c>
+      <c r="H712" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="714" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A714" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B714" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="715" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A715" t="s">
+        <v>4</v>
+      </c>
+      <c r="B715">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="716" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A716" t="s">
         <v>5</v>
       </c>
-      <c r="J711">
-        <v>0.34499999999999997</v>
-      </c>
-      <c r="K711">
-        <v>0.33</v>
-      </c>
-      <c r="L711">
-        <v>0.44</v>
-      </c>
-    </row>
-    <row r="712" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A712" t="s">
-        <v>350</v>
-      </c>
-      <c r="B712">
-        <v>8.4999999999999992E-2</v>
-      </c>
-      <c r="C712" t="s">
-        <v>12</v>
-      </c>
-      <c r="D712" t="s">
-        <v>10</v>
-      </c>
-      <c r="F712" t="s">
-        <v>28</v>
-      </c>
-      <c r="G712" t="s">
-        <v>351</v>
-      </c>
-      <c r="H712" t="s">
-        <v>352</v>
-      </c>
-      <c r="I712">
-        <v>5</v>
-      </c>
-      <c r="J712">
-        <v>8.4999999999999992E-2</v>
-      </c>
-      <c r="K712">
-        <v>8.4999999999999992E-2</v>
-      </c>
-      <c r="L712">
-        <v>0.1127777777777778</v>
-      </c>
-    </row>
-    <row r="713" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A713" t="s">
-        <v>55</v>
-      </c>
-      <c r="B713">
-        <v>1</v>
-      </c>
-      <c r="D713" t="s">
-        <v>10</v>
-      </c>
-      <c r="E713" t="s">
-        <v>56</v>
-      </c>
-      <c r="F713" t="s">
-        <v>57</v>
-      </c>
-      <c r="H713" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="715" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A715" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B715" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="716" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A716" t="s">
-        <v>4</v>
-      </c>
-      <c r="B716">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="717" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B716" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="717" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A717" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B717" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="718" spans="1:13" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="718" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A718" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B718" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="719" spans="1:13" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="719" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A719" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B719" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="720" spans="1:13" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="720" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A720" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B720" t="s">
-        <v>12</v>
+        <v>346</v>
       </c>
     </row>
     <row r="721" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A721" t="s">
+        <v>15</v>
+      </c>
+      <c r="B721" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="722" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A722" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="723" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A723" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B723" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C723" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D723" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E723" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F723" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G723" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H723" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B721" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="722" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A722" t="s">
-        <v>15</v>
-      </c>
-      <c r="B722" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="723" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A723" s="1" t="s">
-        <v>17</v>
+      <c r="I723" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J723" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K723" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L723" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M723" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="724" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A724" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B724" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C724" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D724" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E724" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F724" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G724" s="5" t="s">
+      <c r="A724" t="s">
+        <v>345</v>
+      </c>
+      <c r="B724">
+        <v>1</v>
+      </c>
+      <c r="C724" t="s">
+        <v>12</v>
+      </c>
+      <c r="D724" t="s">
+        <v>10</v>
+      </c>
+      <c r="F724" t="s">
+        <v>26</v>
+      </c>
+      <c r="G724" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="725" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A725" t="s">
+        <v>125</v>
+      </c>
+      <c r="B725">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C725" t="s">
+        <v>12</v>
+      </c>
+      <c r="D725" t="s">
+        <v>10</v>
+      </c>
+      <c r="F725" t="s">
+        <v>28</v>
+      </c>
+      <c r="G725" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H725" t="s">
+        <v>127</v>
+      </c>
+      <c r="I725">
         <v>5</v>
       </c>
-      <c r="H724" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I724" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J724" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K724" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="L724" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M724" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="725" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A725" t="s">
-        <v>353</v>
-      </c>
-      <c r="B725">
-        <v>1</v>
-      </c>
-      <c r="C725" t="s">
-        <v>12</v>
-      </c>
-      <c r="D725" t="s">
-        <v>10</v>
-      </c>
-      <c r="F725" t="s">
-        <v>26</v>
-      </c>
-      <c r="G725" t="s">
-        <v>6</v>
+      <c r="J725" s="43">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="K725">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="L725">
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="726" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A726" t="s">
-        <v>27</v>
+        <v>128</v>
       </c>
       <c r="B726">
-        <v>5.0000000000000002E-11</v>
+        <v>5.0000000000000003E-10</v>
       </c>
       <c r="C726" t="s">
         <v>12</v>
@@ -15087,22 +14888,22 @@
       <c r="I726">
         <v>5</v>
       </c>
-      <c r="J726" s="39">
-        <v>5.0000000000000002E-11</v>
-      </c>
-      <c r="K726" s="39">
-        <v>3.9999999999999998E-11</v>
-      </c>
-      <c r="L726" s="39">
-        <v>6.6666666666666669E-11</v>
+      <c r="J726" s="38">
+        <v>5.0000000000000003E-10</v>
+      </c>
+      <c r="K726">
+        <v>4.0000000000000001E-10</v>
+      </c>
+      <c r="L726" s="38">
+        <v>6.6666666666666664E-10</v>
       </c>
     </row>
     <row r="727" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A727" t="s">
-        <v>31</v>
+        <v>129</v>
       </c>
       <c r="B727">
-        <v>-5.0000000000000002E-11</v>
+        <v>-5.0000000000000003E-10</v>
       </c>
       <c r="C727" t="s">
         <v>12</v>
@@ -15122,14 +14923,14 @@
       <c r="I727">
         <v>5</v>
       </c>
-      <c r="J727" s="39">
-        <v>-5.0000000000000002E-11</v>
-      </c>
-      <c r="K727" s="39">
-        <v>-6.6666666666666669E-11</v>
-      </c>
-      <c r="L727" s="39">
-        <v>-3.9999999999999998E-11</v>
+      <c r="J727">
+        <v>-5.0000000000000003E-10</v>
+      </c>
+      <c r="K727">
+        <v>-6.6666666666666664E-10</v>
+      </c>
+      <c r="L727">
+        <v>-4.0000000000000001E-10</v>
       </c>
       <c r="M727" t="b">
         <v>1</v>
@@ -15137,36 +14938,48 @@
     </row>
     <row r="728" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A728" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="B728">
-        <v>3.4369999999999998</v>
+        <v>0.7</v>
       </c>
       <c r="C728" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="D728" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="F728" t="s">
         <v>28</v>
       </c>
       <c r="G728" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="H728" t="s">
-        <v>36</v>
+        <v>347</v>
+      </c>
+      <c r="I728">
+        <v>5</v>
+      </c>
+      <c r="J728">
+        <v>0.5</v>
+      </c>
+      <c r="K728">
+        <v>0.5</v>
+      </c>
+      <c r="L728">
+        <v>0.7</v>
       </c>
     </row>
     <row r="729" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A729" t="s">
-        <v>37</v>
+        <v>341</v>
       </c>
       <c r="B729">
-        <v>4.0000000000000001E-3</v>
+        <v>0.11018518518518521</v>
       </c>
       <c r="C729" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="D729" t="s">
         <v>10</v>
@@ -15175,307 +14988,355 @@
         <v>28</v>
       </c>
       <c r="G729" t="s">
-        <v>39</v>
+        <v>342</v>
       </c>
       <c r="H729" t="s">
-        <v>36</v>
+        <v>348</v>
+      </c>
+      <c r="I729">
+        <v>5</v>
+      </c>
+      <c r="J729">
+        <v>0.05</v>
+      </c>
+      <c r="K729">
+        <v>0.05</v>
+      </c>
+      <c r="L729">
+        <v>0.11018518518518521</v>
       </c>
     </row>
     <row r="730" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A730" s="40" t="s">
-        <v>40</v>
+      <c r="A730" t="s">
+        <v>55</v>
       </c>
       <c r="B730">
-        <v>3.5000000000000001E-3</v>
-      </c>
-      <c r="C730" t="s">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="D730" t="s">
         <v>10</v>
       </c>
+      <c r="E730" t="s">
+        <v>56</v>
+      </c>
       <c r="F730" t="s">
-        <v>28</v>
-      </c>
-      <c r="G730" s="40" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="H730" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="731" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A731" t="s">
-        <v>43</v>
-      </c>
-      <c r="B731" s="41">
-        <v>-4.0000000000000001E-3</v>
-      </c>
-      <c r="C731" t="s">
-        <v>34</v>
-      </c>
-      <c r="D731" t="s">
-        <v>10</v>
-      </c>
-      <c r="F731" t="s">
-        <v>28</v>
-      </c>
-      <c r="G731" t="s">
-        <v>44</v>
-      </c>
-      <c r="H731" s="42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="732" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A732" t="s">
-        <v>45</v>
-      </c>
-      <c r="B732" s="43">
-        <v>-3.5000000000000001E-3</v>
-      </c>
-      <c r="C732" t="s">
-        <v>41</v>
-      </c>
-      <c r="D732" t="s">
-        <v>10</v>
-      </c>
-      <c r="F732" t="s">
-        <v>28</v>
-      </c>
-      <c r="G732" t="s">
-        <v>46</v>
-      </c>
-      <c r="H732" s="42" t="s">
-        <v>32</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="732" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A732" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B732" s="1" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="733" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A733" t="s">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="B733">
-        <v>0.34499999999999997</v>
-      </c>
-      <c r="C733" t="s">
-        <v>12</v>
-      </c>
-      <c r="D733" t="s">
-        <v>48</v>
-      </c>
-      <c r="F733" t="s">
-        <v>28</v>
-      </c>
-      <c r="G733" t="s">
-        <v>49</v>
-      </c>
-      <c r="H733" t="s">
-        <v>50</v>
-      </c>
-      <c r="I733">
-        <v>5</v>
-      </c>
-      <c r="J733">
-        <v>0.34499999999999997</v>
-      </c>
-      <c r="K733">
-        <v>0.33</v>
-      </c>
-      <c r="L733">
-        <v>0.44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="734" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A734" t="s">
-        <v>350</v>
-      </c>
-      <c r="B734">
-        <v>8.4999999999999992E-2</v>
-      </c>
-      <c r="C734" t="s">
-        <v>12</v>
-      </c>
-      <c r="D734" t="s">
-        <v>10</v>
-      </c>
-      <c r="F734" t="s">
-        <v>28</v>
-      </c>
-      <c r="G734" t="s">
-        <v>351</v>
-      </c>
-      <c r="H734" t="s">
-        <v>352</v>
-      </c>
-      <c r="I734">
         <v>5</v>
       </c>
-      <c r="J734">
-        <v>8.4999999999999992E-2</v>
-      </c>
-      <c r="K734">
-        <v>8.4999999999999992E-2</v>
-      </c>
-      <c r="L734">
-        <v>0.1127777777777778</v>
+      <c r="B734" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="735" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A735" t="s">
-        <v>60</v>
-      </c>
-      <c r="B735">
-        <v>1</v>
-      </c>
-      <c r="C735" t="s">
-        <v>12</v>
-      </c>
-      <c r="D735" t="s">
-        <v>10</v>
-      </c>
-      <c r="F735" t="s">
-        <v>28</v>
-      </c>
-      <c r="G735" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H735" t="s">
-        <v>62</v>
+        <v>7</v>
+      </c>
+      <c r="B735" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="736" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A736" t="s">
-        <v>55</v>
-      </c>
-      <c r="B736">
-        <v>1</v>
-      </c>
-      <c r="D736" t="s">
-        <v>10</v>
-      </c>
-      <c r="E736" t="s">
-        <v>56</v>
-      </c>
-      <c r="F736" t="s">
-        <v>57</v>
-      </c>
-      <c r="H736" t="s">
-        <v>58</v>
+        <v>9</v>
+      </c>
+      <c r="B736" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="737" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A737" t="s">
+        <v>11</v>
+      </c>
+      <c r="B737" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="738" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A738" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B738" s="1" t="s">
-        <v>354</v>
+      <c r="A738" t="s">
+        <v>13</v>
+      </c>
+      <c r="B738" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="739" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A739" t="s">
-        <v>4</v>
-      </c>
-      <c r="B739">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="740" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A740" t="s">
-        <v>5</v>
-      </c>
-      <c r="B740" t="s">
-        <v>6</v>
+        <v>15</v>
+      </c>
+      <c r="B739" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="740" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A740" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="741" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A741" t="s">
+        <v>18</v>
+      </c>
+      <c r="B741" t="s">
+        <v>19</v>
+      </c>
+      <c r="C741" t="s">
+        <v>11</v>
+      </c>
+      <c r="D741" t="s">
+        <v>9</v>
+      </c>
+      <c r="E741" t="s">
+        <v>20</v>
+      </c>
+      <c r="F741" t="s">
         <v>7</v>
       </c>
-      <c r="B741" t="s">
-        <v>8</v>
+      <c r="G741" t="s">
+        <v>5</v>
+      </c>
+      <c r="H741" t="s">
+        <v>13</v>
+      </c>
+      <c r="I741" t="s">
+        <v>21</v>
+      </c>
+      <c r="J741" t="s">
+        <v>22</v>
+      </c>
+      <c r="K741" t="s">
+        <v>23</v>
+      </c>
+      <c r="L741" t="s">
+        <v>24</v>
+      </c>
+      <c r="M741" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="742" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A742" t="s">
-        <v>9</v>
-      </c>
-      <c r="B742" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="743" spans="1:13" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+      <c r="B742">
+        <v>1</v>
+      </c>
+      <c r="C742" t="s">
+        <v>12</v>
+      </c>
+      <c r="D742" t="s">
+        <v>10</v>
+      </c>
+      <c r="F742" t="s">
+        <v>26</v>
+      </c>
+      <c r="G742" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="743" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A743" t="s">
-        <v>11</v>
-      </c>
-      <c r="B743" t="s">
-        <v>12</v>
+        <v>125</v>
+      </c>
+      <c r="B743">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C743" t="s">
+        <v>12</v>
+      </c>
+      <c r="D743" t="s">
+        <v>10</v>
+      </c>
+      <c r="F743" t="s">
+        <v>28</v>
+      </c>
+      <c r="G743" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H743" t="s">
+        <v>36</v>
+      </c>
+      <c r="I743">
+        <v>5</v>
+      </c>
+      <c r="J743">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="K743">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="L743">
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="744" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A744" t="s">
-        <v>13</v>
-      </c>
-      <c r="B744" t="s">
-        <v>355</v>
+        <v>128</v>
+      </c>
+      <c r="B744">
+        <v>5.0000000000000003E-10</v>
+      </c>
+      <c r="C744" t="s">
+        <v>12</v>
+      </c>
+      <c r="D744" t="s">
+        <v>9</v>
+      </c>
+      <c r="F744" t="s">
+        <v>28</v>
+      </c>
+      <c r="G744" t="s">
+        <v>29</v>
+      </c>
+      <c r="H744" t="s">
+        <v>30</v>
+      </c>
+      <c r="I744">
+        <v>5</v>
+      </c>
+      <c r="J744" s="38">
+        <v>5.0000000000000003E-10</v>
+      </c>
+      <c r="K744">
+        <v>4.0000000000000001E-10</v>
+      </c>
+      <c r="L744" s="38">
+        <v>6.6666666666666664E-10</v>
       </c>
     </row>
     <row r="745" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A745" t="s">
-        <v>15</v>
-      </c>
-      <c r="B745" t="s">
-        <v>16</v>
+        <v>129</v>
+      </c>
+      <c r="B745">
+        <v>-5.0000000000000003E-10</v>
+      </c>
+      <c r="C745" t="s">
+        <v>12</v>
+      </c>
+      <c r="D745" t="s">
+        <v>9</v>
+      </c>
+      <c r="F745" t="s">
+        <v>28</v>
+      </c>
+      <c r="G745" t="s">
+        <v>29</v>
+      </c>
+      <c r="H745" t="s">
+        <v>32</v>
+      </c>
+      <c r="I745">
+        <v>5</v>
+      </c>
+      <c r="J745">
+        <v>-5.0000000000000003E-10</v>
+      </c>
+      <c r="K745">
+        <v>-6.6666666666666664E-10</v>
+      </c>
+      <c r="L745">
+        <v>-4.0000000000000001E-10</v>
+      </c>
+      <c r="M745" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="746" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A746" s="1" t="s">
-        <v>17</v>
+      <c r="A746" t="s">
+        <v>47</v>
+      </c>
+      <c r="B746">
+        <v>0.7</v>
+      </c>
+      <c r="C746" t="s">
+        <v>12</v>
+      </c>
+      <c r="D746" t="s">
+        <v>48</v>
+      </c>
+      <c r="F746" t="s">
+        <v>28</v>
+      </c>
+      <c r="G746" t="s">
+        <v>49</v>
+      </c>
+      <c r="H746" t="s">
+        <v>347</v>
+      </c>
+      <c r="I746">
+        <v>5</v>
+      </c>
+      <c r="J746">
+        <v>0.5</v>
+      </c>
+      <c r="K746">
+        <v>0.5</v>
+      </c>
+      <c r="L746">
+        <v>0.7</v>
       </c>
     </row>
     <row r="747" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A747" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B747" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C747" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D747" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E747" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F747" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G747" s="5" t="s">
+      <c r="A747" t="s">
+        <v>341</v>
+      </c>
+      <c r="B747">
+        <v>0.11018518518518521</v>
+      </c>
+      <c r="C747" t="s">
+        <v>12</v>
+      </c>
+      <c r="D747" t="s">
+        <v>10</v>
+      </c>
+      <c r="F747" t="s">
+        <v>28</v>
+      </c>
+      <c r="G747" t="s">
+        <v>342</v>
+      </c>
+      <c r="H747" t="s">
+        <v>348</v>
+      </c>
+      <c r="I747">
         <v>5</v>
       </c>
-      <c r="H747" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I747" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J747" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K747" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="L747" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M747" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="748" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="J747">
+        <v>0.05</v>
+      </c>
+      <c r="K747">
+        <v>0.05</v>
+      </c>
+      <c r="L747">
+        <v>0.11018518518518521</v>
+      </c>
+    </row>
+    <row r="748" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A748" t="s">
-        <v>354</v>
+        <v>60</v>
       </c>
       <c r="B748">
         <v>1</v>
@@ -15487,561 +15348,39 @@
         <v>10</v>
       </c>
       <c r="F748" t="s">
-        <v>26</v>
-      </c>
-      <c r="G748" t="s">
-        <v>6</v>
+        <v>28</v>
+      </c>
+      <c r="G748" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H748" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="749" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A749" t="s">
-        <v>125</v>
+        <v>55</v>
       </c>
       <c r="B749">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C749" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D749" t="s">
         <v>10</v>
       </c>
+      <c r="E749" t="s">
+        <v>56</v>
+      </c>
       <c r="F749" t="s">
-        <v>28</v>
-      </c>
-      <c r="G749" s="2" t="s">
-        <v>126</v>
+        <v>57</v>
       </c>
       <c r="H749" t="s">
-        <v>127</v>
-      </c>
-      <c r="I749">
-        <v>5</v>
-      </c>
-      <c r="J749" s="44">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="K749">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="L749">
-        <v>7.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="750" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A750" t="s">
-        <v>128</v>
-      </c>
-      <c r="B750">
-        <v>5.0000000000000003E-10</v>
-      </c>
-      <c r="C750" t="s">
-        <v>12</v>
-      </c>
-      <c r="D750" t="s">
-        <v>9</v>
-      </c>
-      <c r="F750" t="s">
-        <v>28</v>
-      </c>
-      <c r="G750" t="s">
-        <v>29</v>
-      </c>
-      <c r="H750" t="s">
-        <v>30</v>
-      </c>
-      <c r="I750">
-        <v>5</v>
-      </c>
-      <c r="J750" s="39">
-        <v>5.0000000000000003E-10</v>
-      </c>
-      <c r="K750">
-        <v>4.0000000000000001E-10</v>
-      </c>
-      <c r="L750" s="39">
-        <v>6.6666666666666664E-10</v>
-      </c>
-    </row>
-    <row r="751" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A751" t="s">
-        <v>129</v>
-      </c>
-      <c r="B751">
-        <v>-5.0000000000000003E-10</v>
-      </c>
-      <c r="C751" t="s">
-        <v>12</v>
-      </c>
-      <c r="D751" t="s">
-        <v>9</v>
-      </c>
-      <c r="F751" t="s">
-        <v>28</v>
-      </c>
-      <c r="G751" t="s">
-        <v>29</v>
-      </c>
-      <c r="H751" t="s">
-        <v>32</v>
-      </c>
-      <c r="I751">
-        <v>5</v>
-      </c>
-      <c r="J751">
-        <v>-5.0000000000000003E-10</v>
-      </c>
-      <c r="K751">
-        <v>-6.6666666666666664E-10</v>
-      </c>
-      <c r="L751">
-        <v>-4.0000000000000001E-10</v>
-      </c>
-      <c r="M751" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="752" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A752" t="s">
-        <v>47</v>
-      </c>
-      <c r="B752">
-        <v>0.7</v>
-      </c>
-      <c r="C752" t="s">
-        <v>12</v>
-      </c>
-      <c r="D752" t="s">
-        <v>48</v>
-      </c>
-      <c r="F752" t="s">
-        <v>28</v>
-      </c>
-      <c r="G752" t="s">
-        <v>49</v>
-      </c>
-      <c r="H752" t="s">
-        <v>356</v>
-      </c>
-      <c r="I752">
-        <v>5</v>
-      </c>
-      <c r="J752">
-        <v>0.5</v>
-      </c>
-      <c r="K752">
-        <v>0.5</v>
-      </c>
-      <c r="L752">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="753" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A753" t="s">
-        <v>350</v>
-      </c>
-      <c r="B753">
-        <v>0.11018518518518521</v>
-      </c>
-      <c r="C753" t="s">
-        <v>12</v>
-      </c>
-      <c r="D753" t="s">
-        <v>10</v>
-      </c>
-      <c r="F753" t="s">
-        <v>28</v>
-      </c>
-      <c r="G753" t="s">
-        <v>351</v>
-      </c>
-      <c r="H753" t="s">
-        <v>357</v>
-      </c>
-      <c r="I753">
-        <v>5</v>
-      </c>
-      <c r="J753">
-        <v>0.05</v>
-      </c>
-      <c r="K753">
-        <v>0.05</v>
-      </c>
-      <c r="L753">
-        <v>0.11018518518518521</v>
-      </c>
-    </row>
-    <row r="754" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A754" t="s">
-        <v>55</v>
-      </c>
-      <c r="B754">
-        <v>1</v>
-      </c>
-      <c r="D754" t="s">
-        <v>10</v>
-      </c>
-      <c r="E754" t="s">
-        <v>56</v>
-      </c>
-      <c r="F754" t="s">
-        <v>57</v>
-      </c>
-      <c r="H754" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="756" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A756" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B756" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="757" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A757" t="s">
-        <v>4</v>
-      </c>
-      <c r="B757">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="758" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A758" t="s">
-        <v>5</v>
-      </c>
-      <c r="B758" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="759" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A759" t="s">
-        <v>7</v>
-      </c>
-      <c r="B759" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="760" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A760" t="s">
-        <v>9</v>
-      </c>
-      <c r="B760" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="761" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A761" t="s">
-        <v>11</v>
-      </c>
-      <c r="B761" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="762" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A762" t="s">
-        <v>13</v>
-      </c>
-      <c r="B762" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="763" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A763" t="s">
-        <v>15</v>
-      </c>
-      <c r="B763" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="764" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A764" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="765" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A765" t="s">
-        <v>18</v>
-      </c>
-      <c r="B765" t="s">
-        <v>19</v>
-      </c>
-      <c r="C765" t="s">
-        <v>11</v>
-      </c>
-      <c r="D765" t="s">
-        <v>9</v>
-      </c>
-      <c r="E765" t="s">
-        <v>20</v>
-      </c>
-      <c r="F765" t="s">
-        <v>7</v>
-      </c>
-      <c r="G765" t="s">
-        <v>5</v>
-      </c>
-      <c r="H765" t="s">
-        <v>13</v>
-      </c>
-      <c r="I765" t="s">
-        <v>21</v>
-      </c>
-      <c r="J765" t="s">
-        <v>22</v>
-      </c>
-      <c r="K765" t="s">
-        <v>23</v>
-      </c>
-      <c r="L765" t="s">
-        <v>24</v>
-      </c>
-      <c r="M765" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="766" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A766" t="s">
-        <v>358</v>
-      </c>
-      <c r="B766">
-        <v>1</v>
-      </c>
-      <c r="C766" t="s">
-        <v>12</v>
-      </c>
-      <c r="D766" t="s">
-        <v>10</v>
-      </c>
-      <c r="F766" t="s">
-        <v>26</v>
-      </c>
-      <c r="G766" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="767" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A767" t="s">
-        <v>125</v>
-      </c>
-      <c r="B767">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C767" t="s">
-        <v>12</v>
-      </c>
-      <c r="D767" t="s">
-        <v>10</v>
-      </c>
-      <c r="F767" t="s">
-        <v>28</v>
-      </c>
-      <c r="G767" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H767" t="s">
-        <v>36</v>
-      </c>
-      <c r="I767">
-        <v>5</v>
-      </c>
-      <c r="J767">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="K767">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="L767">
-        <v>7.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="768" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A768" t="s">
-        <v>128</v>
-      </c>
-      <c r="B768">
-        <v>5.0000000000000003E-10</v>
-      </c>
-      <c r="C768" t="s">
-        <v>12</v>
-      </c>
-      <c r="D768" t="s">
-        <v>9</v>
-      </c>
-      <c r="F768" t="s">
-        <v>28</v>
-      </c>
-      <c r="G768" t="s">
-        <v>29</v>
-      </c>
-      <c r="H768" t="s">
-        <v>30</v>
-      </c>
-      <c r="I768">
-        <v>5</v>
-      </c>
-      <c r="J768" s="39">
-        <v>5.0000000000000003E-10</v>
-      </c>
-      <c r="K768">
-        <v>4.0000000000000001E-10</v>
-      </c>
-      <c r="L768" s="39">
-        <v>6.6666666666666664E-10</v>
-      </c>
-    </row>
-    <row r="769" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A769" t="s">
-        <v>129</v>
-      </c>
-      <c r="B769">
-        <v>-5.0000000000000003E-10</v>
-      </c>
-      <c r="C769" t="s">
-        <v>12</v>
-      </c>
-      <c r="D769" t="s">
-        <v>9</v>
-      </c>
-      <c r="F769" t="s">
-        <v>28</v>
-      </c>
-      <c r="G769" t="s">
-        <v>29</v>
-      </c>
-      <c r="H769" t="s">
-        <v>32</v>
-      </c>
-      <c r="I769">
-        <v>5</v>
-      </c>
-      <c r="J769">
-        <v>-5.0000000000000003E-10</v>
-      </c>
-      <c r="K769">
-        <v>-6.6666666666666664E-10</v>
-      </c>
-      <c r="L769">
-        <v>-4.0000000000000001E-10</v>
-      </c>
-      <c r="M769" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="770" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A770" t="s">
-        <v>47</v>
-      </c>
-      <c r="B770">
-        <v>0.7</v>
-      </c>
-      <c r="C770" t="s">
-        <v>12</v>
-      </c>
-      <c r="D770" t="s">
-        <v>48</v>
-      </c>
-      <c r="F770" t="s">
-        <v>28</v>
-      </c>
-      <c r="G770" t="s">
-        <v>49</v>
-      </c>
-      <c r="H770" t="s">
-        <v>356</v>
-      </c>
-      <c r="I770">
-        <v>5</v>
-      </c>
-      <c r="J770">
-        <v>0.5</v>
-      </c>
-      <c r="K770">
-        <v>0.5</v>
-      </c>
-      <c r="L770">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="771" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A771" t="s">
-        <v>350</v>
-      </c>
-      <c r="B771">
-        <v>0.11018518518518521</v>
-      </c>
-      <c r="C771" t="s">
-        <v>12</v>
-      </c>
-      <c r="D771" t="s">
-        <v>10</v>
-      </c>
-      <c r="F771" t="s">
-        <v>28</v>
-      </c>
-      <c r="G771" t="s">
-        <v>351</v>
-      </c>
-      <c r="H771" t="s">
-        <v>357</v>
-      </c>
-      <c r="I771">
-        <v>5</v>
-      </c>
-      <c r="J771">
-        <v>0.05</v>
-      </c>
-      <c r="K771">
-        <v>0.05</v>
-      </c>
-      <c r="L771">
-        <v>0.11018518518518521</v>
-      </c>
-    </row>
-    <row r="772" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A772" t="s">
-        <v>60</v>
-      </c>
-      <c r="B772">
-        <v>1</v>
-      </c>
-      <c r="C772" t="s">
-        <v>12</v>
-      </c>
-      <c r="D772" t="s">
-        <v>10</v>
-      </c>
-      <c r="F772" t="s">
-        <v>28</v>
-      </c>
-      <c r="G772" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H772" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="773" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A773" t="s">
-        <v>55</v>
-      </c>
-      <c r="B773">
-        <v>1</v>
-      </c>
-      <c r="D773" t="s">
-        <v>10</v>
-      </c>
-      <c r="E773" t="s">
-        <v>56</v>
-      </c>
-      <c r="F773" t="s">
-        <v>57</v>
-      </c>
-      <c r="H773" t="s">
-        <v>58</v>
-      </c>
-    </row>
+    <row r="756" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="764" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="767" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="772" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <autoFilter ref="A1:V610" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>